<commit_message>
Added features for HSA Calculations
This update adds two fields to the input spreadsheet: "HSA Contribution" in Column A, and "HSA Eligible" in Row 21. This allows the user to designate which plans are HSA eligible, and how much they would contribute to an HSA if they selected that plan. This eliminates the need for a workaround.
</commit_message>
<xml_diff>
--- a/Health_Monte_Carlo_Input.xlsx
+++ b/Health_Monte_Carlo_Input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/beau/Git/Health_Insurance_Sim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83489A5B-CFDA-4342-8D86-DE064C7187D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D23261ED-BE11-164B-B406-CE7B3812A9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" xr2:uid="{F6F7CCB2-3530-C445-A614-1A88D2B30731}"/>
   </bookViews>
@@ -146,7 +146,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>Issue</t>
   </si>
@@ -259,34 +259,46 @@
     <t>Member "B" Average</t>
   </si>
   <si>
+    <t>Deductible Applying Costs</t>
+  </si>
+  <si>
+    <t>Hit Fam Deductible?</t>
+  </si>
+  <si>
+    <t>Our Cost After Deductible</t>
+  </si>
+  <si>
+    <t>Hit Family OOP Max?</t>
+  </si>
+  <si>
+    <t>Total Costs</t>
+  </si>
+  <si>
+    <t>NonDeductible Costs</t>
+  </si>
+  <si>
+    <t>Total w/ Premium</t>
+  </si>
+  <si>
+    <t>Output Mean</t>
+  </si>
+  <si>
+    <t>Effective Tax Rate</t>
+  </si>
+  <si>
+    <t>HSA Contribution</t>
+  </si>
+  <si>
+    <t>HSA Eligible?</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
     <t>Member "C" Average</t>
-  </si>
-  <si>
-    <t>Deductible Applying Costs</t>
-  </si>
-  <si>
-    <t>Hit Fam Deductible?</t>
-  </si>
-  <si>
-    <t>Our Cost After Deductible</t>
-  </si>
-  <si>
-    <t>Hit Family OOP Max?</t>
-  </si>
-  <si>
-    <t>Total Costs</t>
-  </si>
-  <si>
-    <t>NonDeductible Costs</t>
-  </si>
-  <si>
-    <t>Total w/ Premium</t>
-  </si>
-  <si>
-    <t>Output Mean</t>
-  </si>
-  <si>
-    <t>Effective Tax Rate</t>
   </si>
 </sst>
 </file>
@@ -361,7 +373,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -377,12 +389,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -445,7 +451,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -479,14 +485,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="6" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="6" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="6" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -504,6 +508,19 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="6" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="6" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -825,14 +842,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6844891-A887-1849-A311-9458200AB22B}">
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:S38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.33203125" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.1640625" bestFit="1" customWidth="1"/>
@@ -856,9 +872,9 @@
         <v>36</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G1" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="22" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="17" t="s">
@@ -871,16 +887,16 @@
         <v>5</v>
       </c>
       <c r="K1" s="4"/>
-      <c r="L1" s="24" t="s">
+      <c r="L1" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="24" t="s">
+      <c r="N1" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="24" t="s">
+      <c r="O1" s="22" t="s">
         <v>9</v>
       </c>
     </row>
@@ -891,16 +907,16 @@
       <c r="B2" s="6">
         <v>200</v>
       </c>
-      <c r="C2" s="30">
+      <c r="C2" s="28">
         <v>2</v>
       </c>
-      <c r="D2" s="30">
-        <v>6</v>
-      </c>
-      <c r="E2" s="30">
-        <v>12</v>
-      </c>
-      <c r="F2" s="33"/>
+      <c r="D2" s="28">
+        <v>2</v>
+      </c>
+      <c r="E2" s="28">
+        <v>4</v>
+      </c>
+      <c r="F2" s="31"/>
       <c r="G2" s="7">
         <v>0.2</v>
       </c>
@@ -934,16 +950,16 @@
       <c r="B3" s="6">
         <v>400</v>
       </c>
-      <c r="C3" s="30">
+      <c r="C3" s="28">
         <v>1</v>
       </c>
-      <c r="D3" s="30">
-        <v>3</v>
-      </c>
-      <c r="E3" s="30">
-        <v>6</v>
-      </c>
-      <c r="F3" s="33"/>
+      <c r="D3" s="28">
+        <v>1</v>
+      </c>
+      <c r="E3" s="28">
+        <v>4</v>
+      </c>
+      <c r="F3" s="31"/>
       <c r="G3" s="7">
         <v>0.2</v>
       </c>
@@ -977,16 +993,16 @@
       <c r="B4" s="11">
         <v>235</v>
       </c>
-      <c r="C4" s="30">
-        <v>0</v>
-      </c>
-      <c r="D4" s="30">
-        <v>0</v>
-      </c>
-      <c r="E4" s="30">
-        <v>0</v>
-      </c>
-      <c r="F4" s="33"/>
+      <c r="C4" s="28">
+        <v>0</v>
+      </c>
+      <c r="D4" s="28">
+        <v>0</v>
+      </c>
+      <c r="E4" s="28">
+        <v>0</v>
+      </c>
+      <c r="F4" s="31"/>
       <c r="G4" s="7">
         <v>0.4</v>
       </c>
@@ -1020,16 +1036,16 @@
       <c r="B5" s="11">
         <v>120</v>
       </c>
-      <c r="C5" s="30">
-        <v>0</v>
-      </c>
-      <c r="D5" s="30">
-        <v>4.5</v>
-      </c>
-      <c r="E5" s="30">
-        <v>0</v>
-      </c>
-      <c r="F5" s="33"/>
+      <c r="C5" s="28">
+        <v>0</v>
+      </c>
+      <c r="D5" s="28">
+        <v>3</v>
+      </c>
+      <c r="E5" s="28">
+        <v>0</v>
+      </c>
+      <c r="F5" s="31"/>
       <c r="G5" s="7">
         <v>0.2</v>
       </c>
@@ -1063,16 +1079,16 @@
       <c r="B6" s="11">
         <v>20</v>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="28">
         <v>2</v>
       </c>
-      <c r="D6" s="30">
-        <v>3</v>
-      </c>
-      <c r="E6" s="30">
-        <v>4</v>
-      </c>
-      <c r="F6" s="33"/>
+      <c r="D6" s="28">
+        <v>2</v>
+      </c>
+      <c r="E6" s="28">
+        <v>1</v>
+      </c>
+      <c r="F6" s="31"/>
       <c r="G6" s="7">
         <v>0.2</v>
       </c>
@@ -1106,16 +1122,16 @@
       <c r="B7" s="11">
         <v>100</v>
       </c>
-      <c r="C7" s="30">
+      <c r="C7" s="28">
         <v>0.5</v>
       </c>
-      <c r="D7" s="30">
-        <v>2</v>
-      </c>
-      <c r="E7" s="30">
-        <v>2</v>
-      </c>
-      <c r="F7" s="33"/>
+      <c r="D7" s="28">
+        <v>1</v>
+      </c>
+      <c r="E7" s="28">
+        <v>1</v>
+      </c>
+      <c r="F7" s="31"/>
       <c r="G7" s="7">
         <v>0.2</v>
       </c>
@@ -1149,16 +1165,16 @@
       <c r="B8" s="11">
         <v>250</v>
       </c>
-      <c r="C8" s="30">
-        <v>0</v>
-      </c>
-      <c r="D8" s="30">
+      <c r="C8" s="28">
+        <v>0</v>
+      </c>
+      <c r="D8" s="28">
         <v>1</v>
       </c>
-      <c r="E8" s="30">
-        <v>0</v>
-      </c>
-      <c r="F8" s="33"/>
+      <c r="E8" s="28">
+        <v>0</v>
+      </c>
+      <c r="F8" s="31"/>
       <c r="G8" s="7">
         <v>0.2</v>
       </c>
@@ -1192,16 +1208,16 @@
       <c r="B9" s="11">
         <v>300</v>
       </c>
-      <c r="C9" s="30">
+      <c r="C9" s="28">
         <v>2</v>
       </c>
-      <c r="D9" s="30">
-        <v>4</v>
-      </c>
-      <c r="E9" s="30">
-        <v>4</v>
-      </c>
-      <c r="F9" s="33"/>
+      <c r="D9" s="28">
+        <v>2</v>
+      </c>
+      <c r="E9" s="28">
+        <v>3</v>
+      </c>
+      <c r="F9" s="31"/>
       <c r="G9" s="7">
         <v>0.2</v>
       </c>
@@ -1235,16 +1251,16 @@
       <c r="B10" s="11">
         <v>3500</v>
       </c>
-      <c r="C10" s="30">
+      <c r="C10" s="28">
         <v>1</v>
       </c>
-      <c r="D10" s="30">
-        <v>2</v>
-      </c>
-      <c r="E10" s="30">
-        <v>2</v>
-      </c>
-      <c r="F10" s="33"/>
+      <c r="D10" s="28">
+        <v>1</v>
+      </c>
+      <c r="E10" s="28">
+        <v>1</v>
+      </c>
+      <c r="F10" s="31"/>
       <c r="G10" s="7">
         <v>0.2</v>
       </c>
@@ -1278,16 +1294,16 @@
       <c r="B11" s="11">
         <v>200</v>
       </c>
-      <c r="C11" s="30">
+      <c r="C11" s="28">
         <v>1</v>
       </c>
-      <c r="D11" s="30">
-        <v>2</v>
-      </c>
-      <c r="E11" s="30">
-        <v>0</v>
-      </c>
-      <c r="F11" s="33"/>
+      <c r="D11" s="28">
+        <v>1</v>
+      </c>
+      <c r="E11" s="28">
+        <v>1</v>
+      </c>
+      <c r="F11" s="31"/>
       <c r="G11" s="7">
         <v>0.2</v>
       </c>
@@ -1321,16 +1337,16 @@
       <c r="B12" s="11">
         <v>25000</v>
       </c>
-      <c r="C12" s="30">
-        <v>0</v>
-      </c>
-      <c r="D12" s="30">
-        <v>0</v>
-      </c>
-      <c r="E12" s="30">
-        <v>0</v>
-      </c>
-      <c r="F12" s="33"/>
+      <c r="C12" s="28">
+        <v>0</v>
+      </c>
+      <c r="D12" s="28">
+        <v>0</v>
+      </c>
+      <c r="E12" s="28">
+        <v>0</v>
+      </c>
+      <c r="F12" s="31"/>
       <c r="G12" s="7">
         <v>0.2</v>
       </c>
@@ -1364,16 +1380,16 @@
       <c r="B13" s="11">
         <v>50000</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="29">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="D13" s="31">
+      <c r="D13" s="29">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="29">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="F13" s="33"/>
+      <c r="F13" s="31"/>
       <c r="G13" s="7">
         <v>0.2</v>
       </c>
@@ -1407,16 +1423,16 @@
       <c r="B14" s="15">
         <v>15000</v>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="30">
         <v>0.01</v>
       </c>
-      <c r="D14" s="32">
+      <c r="D14" s="30">
         <v>0.01</v>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="30">
         <v>0.01</v>
       </c>
-      <c r="F14" s="33"/>
+      <c r="F14" s="31"/>
       <c r="G14" s="7">
         <v>0.2</v>
       </c>
@@ -1455,13 +1471,14 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="29">
-        <v>0</v>
-      </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
+        <v>45</v>
+      </c>
+      <c r="B16" s="27">
+        <v>0.24</v>
+      </c>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
       <c r="F16" t="s">
         <v>23</v>
       </c>
@@ -1500,6 +1517,12 @@
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="23">
+        <v>8550</v>
+      </c>
       <c r="F17" t="s">
         <v>25</v>
       </c>
@@ -1547,23 +1570,24 @@
       <c r="J18" s="17">
         <v>1500</v>
       </c>
-      <c r="L18" s="17">
+      <c r="K18" s="37"/>
+      <c r="L18" s="38">
         <v>3000</v>
       </c>
-      <c r="M18" s="17">
+      <c r="M18" s="38">
         <v>8550</v>
       </c>
-      <c r="N18" s="17">
+      <c r="N18" s="38">
         <v>8550</v>
       </c>
-      <c r="O18" s="17">
+      <c r="O18" s="38">
         <v>8550</v>
       </c>
       <c r="Q18" s="16"/>
       <c r="S18" s="4"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="24" t="s">
         <v>30</v>
       </c>
       <c r="F19" t="s">
@@ -1581,17 +1605,17 @@
       <c r="J19" s="17">
         <v>1000</v>
       </c>
-      <c r="K19" s="19"/>
-      <c r="L19" s="20">
+      <c r="K19" s="39"/>
+      <c r="L19" s="38">
         <v>1000</v>
       </c>
-      <c r="M19" s="20">
+      <c r="M19" s="38">
         <v>2500</v>
       </c>
-      <c r="N19" s="20">
+      <c r="N19" s="38">
         <v>7500</v>
       </c>
-      <c r="O19" s="20">
+      <c r="O19" s="38">
         <v>9700</v>
       </c>
       <c r="P19" s="8"/>
@@ -1600,12 +1624,13 @@
       <c r="A20" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="27" cm="1">
+      <c r="B20" s="25" cm="1">
         <f t="array" ref="B20">SUMPRODUCT(B2:B14*(C2:E14))</f>
-        <v>31720</v>
-      </c>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
+        <v>19360</v>
+      </c>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
       <c r="F20" t="s">
         <v>26</v>
       </c>
@@ -1621,546 +1646,580 @@
       <c r="J20" s="17">
         <v>3000</v>
       </c>
-      <c r="K20" s="19"/>
-      <c r="L20" s="20">
+      <c r="K20" s="39"/>
+      <c r="L20" s="38">
         <v>6000</v>
       </c>
-      <c r="M20" s="20">
+      <c r="M20" s="38">
         <v>17100</v>
       </c>
-      <c r="N20" s="20">
+      <c r="N20" s="38">
         <v>17100</v>
       </c>
-      <c r="O20" s="20">
+      <c r="O20" s="38">
         <v>9700</v>
       </c>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K21" s="40"/>
+      <c r="L21" s="41" t="s">
+        <v>49</v>
+      </c>
+      <c r="M21" s="42"/>
+      <c r="N21" s="41" t="s">
+        <v>49</v>
+      </c>
+      <c r="O21" s="41" t="s">
+        <v>48</v>
+      </c>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="F22" s="26" t="s">
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="17"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="F23" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="P22" s="4"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="F23" t="s">
+      <c r="I23" s="23">
+        <f>I16</f>
+        <v>5856</v>
+      </c>
+      <c r="M23" s="23">
+        <f>M16</f>
+        <v>9957.6959999999999</v>
+      </c>
+      <c r="P23" s="4"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="F24" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="25">
+      <c r="G24" s="23">
         <f>G16</f>
         <v>3276</v>
       </c>
-      <c r="H23" s="25">
+      <c r="H24" s="23">
         <f>H16</f>
         <v>3996</v>
       </c>
-      <c r="I23" s="25">
-        <f>I16</f>
-        <v>5856</v>
-      </c>
-      <c r="J23" s="25">
+      <c r="I24" s="23">
+        <f>SUM(I16,I20)</f>
+        <v>17856</v>
+      </c>
+      <c r="J24" s="23">
         <f>J16</f>
         <v>9312</v>
       </c>
-      <c r="L23" s="25">
+      <c r="L24" s="23">
         <f>L16</f>
         <v>12157.823999999997</v>
       </c>
-      <c r="M23" s="25">
-        <f>M16</f>
-        <v>9957.6959999999999</v>
-      </c>
-      <c r="N23" s="25">
+      <c r="M24" s="23">
+        <f>SUM(M16,M20)</f>
+        <v>27057.696</v>
+      </c>
+      <c r="N24" s="23">
         <f>N16</f>
         <v>8191.8479999999981</v>
       </c>
-      <c r="O23" s="25">
+      <c r="O24" s="23">
         <f>O16</f>
         <v>8261.9880000000012</v>
       </c>
-      <c r="P23" s="21"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="F24" t="s">
+      <c r="P24" s="19"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="F25" t="s">
         <v>28</v>
       </c>
-      <c r="G24" s="25">
+      <c r="G25" s="23">
         <f>SUM(G16,G20)</f>
         <v>15276</v>
       </c>
-      <c r="H24" s="25">
+      <c r="H25" s="23">
         <f>SUM(H16,H20)</f>
         <v>17996</v>
       </c>
-      <c r="I24" s="25">
-        <f>SUM(I16,I20)</f>
-        <v>17856</v>
-      </c>
-      <c r="J24" s="25">
+      <c r="I25" s="12">
+        <v>17906</v>
+      </c>
+      <c r="J25" s="23">
         <f>SUM(J16,J20)</f>
         <v>12312</v>
       </c>
-      <c r="L24" s="25">
+      <c r="L25" s="23">
         <f>SUM(L16,L20)</f>
         <v>18157.823999999997</v>
       </c>
-      <c r="M24" s="25">
-        <f>SUM(M16,M20)</f>
-        <v>27057.696</v>
-      </c>
-      <c r="N24" s="25">
+      <c r="M25">
+        <v>24223</v>
+      </c>
+      <c r="N25" s="23">
         <f>SUM(N16,N20)</f>
         <v>25291.847999999998</v>
       </c>
-      <c r="O24" s="25">
+      <c r="O25" s="23">
         <f>SUM(O16,O20)</f>
         <v>17961.988000000001</v>
       </c>
-      <c r="P24" s="21"/>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="F25" s="28" t="s">
+      <c r="P25" s="19"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="F26" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="G25">
+      <c r="G26">
         <v>15976</v>
       </c>
-      <c r="H25">
+      <c r="H26">
         <v>18056</v>
       </c>
-      <c r="I25" s="12">
-        <v>17906</v>
-      </c>
-      <c r="J25">
-        <v>12512</v>
-      </c>
-      <c r="L25">
-        <v>18407</v>
-      </c>
-      <c r="M25">
-        <v>24223</v>
-      </c>
-      <c r="N25">
-        <v>23835</v>
-      </c>
-      <c r="O25">
-        <v>17022</v>
-      </c>
-      <c r="P25" s="12"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="F26" t="s">
-        <v>34</v>
-      </c>
-      <c r="G26" s="25">
-        <f>G24-G25</f>
-        <v>-700</v>
-      </c>
-      <c r="H26" s="25">
-        <f>H24-H25</f>
-        <v>-60</v>
-      </c>
-      <c r="I26" s="25">
+      <c r="I26" s="23">
         <f>I24-I25</f>
         <v>-50</v>
       </c>
-      <c r="J26" s="25">
-        <f>J24-J25</f>
-        <v>-200</v>
-      </c>
-      <c r="L26" s="25">
-        <f>L24-L25</f>
-        <v>-249.17600000000311</v>
-      </c>
-      <c r="M26" s="25">
+      <c r="J26">
+        <v>12512</v>
+      </c>
+      <c r="L26">
+        <v>18407</v>
+      </c>
+      <c r="M26" s="23">
         <f>M24-M25</f>
         <v>2834.6959999999999</v>
       </c>
-      <c r="N26" s="25">
-        <f>N24-N25</f>
+      <c r="N26">
+        <v>23835</v>
+      </c>
+      <c r="O26">
+        <v>17022</v>
+      </c>
+      <c r="P26" s="12"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="F27" t="s">
+        <v>34</v>
+      </c>
+      <c r="G27" s="23">
+        <f>G25-G26</f>
+        <v>-700</v>
+      </c>
+      <c r="H27" s="23">
+        <f>H25-H26</f>
+        <v>-60</v>
+      </c>
+      <c r="I27" s="23">
+        <f>I16/12</f>
+        <v>488</v>
+      </c>
+      <c r="J27" s="23">
+        <f>J25-J26</f>
+        <v>-200</v>
+      </c>
+      <c r="L27" s="23">
+        <f>L25-L26</f>
+        <v>-249.17600000000311</v>
+      </c>
+      <c r="M27" s="23">
+        <f>M16/12</f>
+        <v>829.80799999999999</v>
+      </c>
+      <c r="N27" s="23">
+        <f>N25-N26</f>
         <v>1456.8479999999981</v>
       </c>
-      <c r="O26" s="25">
-        <f>O24-O25</f>
+      <c r="O27" s="23">
+        <f>O25-O26</f>
         <v>939.98800000000119</v>
       </c>
-      <c r="P26" s="22"/>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="G27" s="25">
+      <c r="P27" s="20"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="G28" s="23">
         <f>G16/12</f>
         <v>273</v>
       </c>
-      <c r="H27" s="25">
+      <c r="H28" s="23">
         <f>H16/12</f>
         <v>333</v>
       </c>
-      <c r="I27" s="25">
-        <f>I16/12</f>
-        <v>488</v>
-      </c>
-      <c r="J27" s="25">
+      <c r="I28" s="23" cm="1">
+        <f t="array" ref="I28">SUMPRODUCT(I2:I3*(InputParms!$C$2:$D$3))+SUMPRODUCT(I5:I10*(InputParms!$C$5:$D$10))</f>
+        <v>1352.5</v>
+      </c>
+      <c r="J28" s="23">
         <f>J16/12</f>
         <v>776</v>
       </c>
-      <c r="L27" s="25">
+      <c r="L28" s="23">
         <f>L16/12</f>
         <v>1013.1519999999997</v>
       </c>
-      <c r="M27" s="25">
-        <f>M16/12</f>
-        <v>829.80799999999999</v>
-      </c>
-      <c r="N27" s="25">
+      <c r="M28" s="17" cm="1">
+        <f t="array" ref="M28">SUMPRODUCT(M2:M3*(InputParms!$C$2:$D$3))+SUMPRODUCT(M5:M7*(InputParms!$C$5:$D$7))+SUMPRODUCT(M9:M10*(InputParms!$C$9:$D$10))</f>
+        <v>1415</v>
+      </c>
+      <c r="N28" s="23">
         <f>N16/12</f>
         <v>682.65399999999988</v>
       </c>
-      <c r="O27" s="25">
+      <c r="O28" s="23">
         <f>O16/12</f>
         <v>688.49900000000014</v>
       </c>
-      <c r="P27" s="23"/>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="F28" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" s="25">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="25" cm="1">
-        <f t="array" ref="H28">SUMPRODUCT(H2:H3*($C$2:$E$3))+SUMPRODUCT(H5:H10*($C$5:$E$10))</f>
-        <v>3982.5</v>
-      </c>
-      <c r="I28" s="25" cm="1">
-        <f t="array" ref="I28">SUMPRODUCT(I2:I3*($C$2:$E$3))+SUMPRODUCT(I5:I10*($C$5:$E$10))</f>
-        <v>3637.5</v>
-      </c>
-      <c r="J28" s="17" cm="1">
-        <f t="array" ref="J28">SUMPRODUCT(J2:J3*($C$2:$E$3))+SUMPRODUCT(J5:J10*($C$5:$E$10))</f>
-        <v>3387.5</v>
-      </c>
-      <c r="L28" s="17" cm="1">
-        <f t="array" ref="L28">SUMPRODUCT(L2:L3*($C$2:$E$3))+SUMPRODUCT(L5:L7*($C$5:$E$7))+SUMPRODUCT(L9:L10*($C$9:$E$10))</f>
-        <v>2592</v>
-      </c>
-      <c r="M28" s="17" cm="1">
-        <f t="array" ref="M28">SUMPRODUCT(M2:M3*($C$2:$E$3))+SUMPRODUCT(M5:M7*($C$5:$E$7))+SUMPRODUCT(M9:M10*($C$9:$E$10))</f>
-        <v>4085</v>
-      </c>
-      <c r="N28" s="17" cm="1">
-        <f t="array" ref="N28">SUMPRODUCT(N2:N3*($C$2:$E$3))+SUMPRODUCT(N5:N7*($C$5:$E$7))+SUMPRODUCT(N9:N10*($C$9:$E$10))</f>
-        <v>4765</v>
-      </c>
-      <c r="O28" s="25">
-        <f>0</f>
-        <v>0</v>
-      </c>
-      <c r="P28" s="23"/>
+      <c r="P28" s="21"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="F29" t="s">
-        <v>38</v>
-      </c>
-      <c r="G29" s="37" cm="1">
-        <f t="array" ref="G29">SUMPRODUCT($B$2:$B$14*($C$2:$E$14))</f>
-        <v>31720</v>
-      </c>
-      <c r="H29" s="35" cm="1">
-        <f t="array" ref="H29">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))</f>
-        <v>1800</v>
-      </c>
-      <c r="I29" s="35" cm="1">
-        <f t="array" ref="I29">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))</f>
-        <v>1800</v>
-      </c>
-      <c r="J29" s="22" cm="1">
-        <f t="array" ref="J29">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))</f>
-        <v>1800</v>
-      </c>
-      <c r="L29" s="22" cm="1">
-        <f t="array" ref="L29">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))+SUMPRODUCT($B$8*($C$8:$E$8))</f>
-        <v>2050</v>
-      </c>
-      <c r="M29" s="22" cm="1">
-        <f t="array" ref="M29">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))+SUMPRODUCT($B$8*($C$8:$E$8))</f>
-        <v>2050</v>
-      </c>
-      <c r="N29" s="22" cm="1">
-        <f t="array" ref="N29">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))+SUMPRODUCT($B$8*($C$8:$E$8))</f>
-        <v>2050</v>
-      </c>
-      <c r="O29" s="37" cm="1">
-        <f t="array" ref="O29">SUMPRODUCT($B$2:$B$14*($C$2:$E$14))</f>
-        <v>31720</v>
-      </c>
-      <c r="P29" s="22"/>
+        <v>42</v>
+      </c>
+      <c r="G29" s="23">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="23" cm="1">
+        <f t="array" ref="H29">SUMPRODUCT(H2:H3*($C$2:$E$3))+SUMPRODUCT(H5:H10*($C$5:$E$10))</f>
+        <v>2362.5</v>
+      </c>
+      <c r="I29" s="33" cm="1">
+        <f t="array" ref="I29">SUMPRODUCT(InputParms!$B$4*(InputParms!$C$4:$D$4))+SUMPRODUCT(InputParms!$B$11:$B$14*(InputParms!$C$11:$D$14))</f>
+        <v>1200</v>
+      </c>
+      <c r="J29" s="17" cm="1">
+        <f t="array" ref="J29">SUMPRODUCT(J2:J3*($C$2:$E$3))+SUMPRODUCT(J5:J10*($C$5:$E$10))</f>
+        <v>2012.5</v>
+      </c>
+      <c r="L29" s="17" cm="1">
+        <f t="array" ref="L29">SUMPRODUCT(L2:L3*($C$2:$E$3))+SUMPRODUCT(L5:L7*($C$5:$E$7))+SUMPRODUCT(L9:L10*($C$9:$E$10))</f>
+        <v>1505</v>
+      </c>
+      <c r="M29" s="20" cm="1">
+        <f t="array" ref="M29">SUMPRODUCT(InputParms!$B$4*(InputParms!$C$4:$D$4))+SUMPRODUCT(InputParms!$B$11:$B$14*(InputParms!$C$11:$D$14))+SUMPRODUCT(InputParms!$B$8*(InputParms!$C$8:$D$8))</f>
+        <v>1450</v>
+      </c>
+      <c r="N29" s="17" cm="1">
+        <f t="array" ref="N29">SUMPRODUCT(N2:N3*($C$2:$E$3))+SUMPRODUCT(N5:N7*($C$5:$E$7))+SUMPRODUCT(N9:N10*($C$9:$E$10))</f>
+        <v>2755</v>
+      </c>
+      <c r="O29" s="23">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="P29" s="21"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="F30" t="s">
-        <v>39</v>
-      </c>
-      <c r="G30" t="b">
-        <f>G29&gt;G19</f>
-        <v>1</v>
-      </c>
-      <c r="H30" t="b">
-        <f>H29&gt;H19</f>
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="G30" s="35" cm="1">
+        <f t="array" ref="G30">SUMPRODUCT($B$2:$B$14*($C$2:$E$14))</f>
+        <v>19360</v>
+      </c>
+      <c r="H30" s="33" cm="1">
+        <f t="array" ref="H30">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))</f>
+        <v>1800</v>
       </c>
       <c r="I30" t="b">
         <f>I29&gt;I19</f>
         <v>0</v>
       </c>
-      <c r="J30" s="12" t="b">
-        <f>J29&gt;J19</f>
-        <v>1</v>
-      </c>
-      <c r="L30" s="12" t="b">
-        <f>L29&gt;L19</f>
-        <v>1</v>
+      <c r="J30" s="20" cm="1">
+        <f t="array" ref="J30">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))</f>
+        <v>1800</v>
+      </c>
+      <c r="L30" s="20" cm="1">
+        <f t="array" ref="L30">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))+SUMPRODUCT($B$8*($C$8:$E$8))</f>
+        <v>2050</v>
       </c>
       <c r="M30" s="12" t="b">
         <f>M29&gt;M19</f>
         <v>0</v>
       </c>
-      <c r="N30" s="12" t="b">
-        <f>N29&gt;N19</f>
-        <v>0</v>
-      </c>
-      <c r="O30" t="b">
-        <f>O29&gt;O19</f>
-        <v>1</v>
-      </c>
-      <c r="P30" s="22"/>
+      <c r="N30" s="20" cm="1">
+        <f t="array" ref="N30">SUMPRODUCT($B$4*($C$4:$E$4))+SUMPRODUCT($B$11:$B$14*($C$11:$E$14))+SUMPRODUCT($B$8*($C$8:$E$8))</f>
+        <v>2050</v>
+      </c>
+      <c r="O30" s="35" cm="1">
+        <f t="array" ref="O30">SUMPRODUCT($B$2:$B$14*($C$2:$E$14))</f>
+        <v>19360</v>
+      </c>
+      <c r="P30" s="20"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="F31" t="s">
-        <v>40</v>
-      </c>
-      <c r="G31" s="34">
-        <f>IF(G30,(G29-G19)*AVERAGE(G2:G14),0)</f>
-        <v>5453.5384615384619</v>
-      </c>
-      <c r="H31" s="34">
-        <f>IF(H30,(H29-H19)*AVERAGE(H4,H11:H14),0)</f>
-        <v>0</v>
-      </c>
-      <c r="I31" s="34">
+        <v>38</v>
+      </c>
+      <c r="G31" t="b">
+        <f>G30&gt;G19</f>
+        <v>1</v>
+      </c>
+      <c r="H31" t="b">
+        <f>H30&gt;H19</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="32">
         <f>IF(I30,(I29-I19)*AVERAGE(I4,I11:I14),0)</f>
         <v>0</v>
       </c>
-      <c r="J31" s="36">
-        <f>IF(J30,(J29-J19)*AVERAGE(J4,J11:J14),0)</f>
-        <v>207.99999999999997</v>
-      </c>
-      <c r="L31" s="36">
-        <f>IF(L30,(L29-L19)*AVERAGE(L4,L11:L14,L8),0)</f>
-        <v>236.25</v>
-      </c>
-      <c r="M31" s="36">
+      <c r="J31" s="12" t="b">
+        <f>J30&gt;J19</f>
+        <v>1</v>
+      </c>
+      <c r="L31" s="12" t="b">
+        <f>L30&gt;L19</f>
+        <v>1</v>
+      </c>
+      <c r="M31" s="34">
         <f>IF(M30,(M29-M19)*AVERAGE(M4,M11:M14,M8),0)</f>
         <v>0</v>
       </c>
-      <c r="N31" s="36">
-        <f>IF(N30,(N29-N19)*AVERAGE(N4,N11:N14,N8),0)</f>
-        <v>0</v>
-      </c>
-      <c r="O31" s="34">
-        <f>IF(O30,(O29-O19)*AVERAGE(O2:O14),0)</f>
-        <v>846.92307692307702</v>
-      </c>
-      <c r="P31" s="12"/>
+      <c r="N31" s="12" t="b">
+        <f>N30&gt;N19</f>
+        <v>0</v>
+      </c>
+      <c r="O31" t="b">
+        <f>O30&gt;O19</f>
+        <v>1</v>
+      </c>
+      <c r="P31" s="20"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="F32" t="s">
-        <v>41</v>
-      </c>
-      <c r="G32" t="b">
-        <f>IF(G30,G31+G19&gt;G20,G29&gt;G20)</f>
-        <v>0</v>
-      </c>
-      <c r="H32" t="b">
-        <f>IF(H30,H31+H19&gt;H20,H29&gt;H20)</f>
+        <v>39</v>
+      </c>
+      <c r="G32" s="32">
+        <f>IF(G31,(G30-G19)*AVERAGE(G2:G14),0)</f>
+        <v>2791.3846153846157</v>
+      </c>
+      <c r="H32" s="32">
+        <f>IF(H31,(H30-H19)*AVERAGE(H4,H11:H14),0)</f>
         <v>0</v>
       </c>
       <c r="I32" t="b">
         <f>IF(I30,I31+I19&gt;I20,I29&gt;I20)</f>
         <v>0</v>
       </c>
-      <c r="J32" s="12" t="b">
-        <f>IF(J30,J31+J19&gt;J20,J29&gt;J20)</f>
-        <v>0</v>
-      </c>
-      <c r="L32" s="12" t="b">
-        <f>IF(L30,L31+L19&gt;L20,L29&gt;L20)</f>
-        <v>0</v>
+      <c r="J32" s="34">
+        <f>IF(J31,(J30-J19)*AVERAGE(J4,J11:J14),0)</f>
+        <v>207.99999999999997</v>
+      </c>
+      <c r="L32" s="34">
+        <f>IF(L31,(L30-L19)*AVERAGE(L4,L11:L14,L8),0)</f>
+        <v>236.25</v>
       </c>
       <c r="M32" s="12" t="b">
         <f>IF(M30,M31+M19&gt;M20,M29&gt;M20)</f>
         <v>0</v>
       </c>
-      <c r="N32" s="12" t="b">
-        <f>IF(N30,N31+N19&gt;N20,N29&gt;N20)</f>
-        <v>0</v>
-      </c>
-      <c r="O32" t="b">
-        <f>IF(O30,O31+O19&gt;O20,O29&gt;O20)</f>
-        <v>1</v>
-      </c>
-      <c r="P32" s="4"/>
+      <c r="N32" s="34">
+        <f>IF(N31,(N30-N19)*AVERAGE(N4,N11:N14,N8),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O32" s="32">
+        <f>IF(O31,(O30-O19)*AVERAGE(O2:O14),0)</f>
+        <v>371.53846153846155</v>
+      </c>
+      <c r="P32" s="12"/>
     </row>
     <row r="33" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F33" t="s">
-        <v>42</v>
-      </c>
-      <c r="G33" s="34">
-        <f>IF(G32,G20,IF(G30,G31+G19,G29))+G28</f>
-        <v>11853.538461538461</v>
-      </c>
-      <c r="H33" s="34">
-        <f>IF(H32,H20,IF(H30,H31+H19,H29))+H28</f>
-        <v>5782.5</v>
-      </c>
-      <c r="I33" s="34">
+        <v>40</v>
+      </c>
+      <c r="G33" t="b">
+        <f>IF(G31,G32+G19&gt;G20,G30&gt;G20)</f>
+        <v>0</v>
+      </c>
+      <c r="H33" t="b">
+        <f>IF(H31,H32+H19&gt;H20,H30&gt;H20)</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="32">
         <f>IF(I32,I20,IF(I30,I31+I19,I29))+I28</f>
-        <v>5437.5</v>
-      </c>
-      <c r="J33" s="36">
-        <f>IF(J32,J20,IF(J30,J31+J19,J29))+J28</f>
-        <v>4595.5</v>
-      </c>
-      <c r="L33" s="36">
-        <f>IF(L32,L20,IF(L30,L31+L19,L29))+L28</f>
-        <v>3828.25</v>
-      </c>
-      <c r="M33" s="36">
+        <v>2552.5</v>
+      </c>
+      <c r="J33" s="12" t="b">
+        <f>IF(J31,J32+J19&gt;J20,J30&gt;J20)</f>
+        <v>0</v>
+      </c>
+      <c r="L33" s="12" t="b">
+        <f>IF(L31,L32+L19&gt;L20,L30&gt;L20)</f>
+        <v>0</v>
+      </c>
+      <c r="M33" s="34">
         <f>IF(M32,M20,IF(M30,M31+M19,M29))+M28</f>
-        <v>6135</v>
-      </c>
-      <c r="N33" s="36">
-        <f>IF(N32,N20,IF(N30,N31+N19,N29))+N28</f>
-        <v>6815</v>
-      </c>
-      <c r="O33" s="34">
-        <f>IF(O32,O20,IF(O30,O31+O19,O29))+O28</f>
-        <v>9700</v>
-      </c>
-      <c r="P33" s="22"/>
+        <v>2865</v>
+      </c>
+      <c r="N33" s="12" t="b">
+        <f>IF(N31,N32+N19&gt;N20,N30&gt;N20)</f>
+        <v>0</v>
+      </c>
+      <c r="O33" t="b">
+        <f>IF(O31,O32+O19&gt;O20,O30&gt;O20)</f>
+        <v>1</v>
+      </c>
+      <c r="P33" s="4"/>
     </row>
     <row r="34" spans="6:16" x14ac:dyDescent="0.2">
       <c r="F34" t="s">
-        <v>44</v>
-      </c>
-      <c r="G34" s="25">
-        <f>G33+G16</f>
-        <v>15129.538461538461</v>
-      </c>
-      <c r="H34" s="25">
-        <f>H33+H16</f>
-        <v>9778.5</v>
-      </c>
-      <c r="I34" s="25">
+        <v>41</v>
+      </c>
+      <c r="G34" s="32">
+        <f>IF(G33,G20,IF(G31,G32+G19,G30))+G29</f>
+        <v>9191.3846153846152</v>
+      </c>
+      <c r="H34" s="32">
+        <f>IF(H33,H20,IF(H31,H32+H19,H30))+H29</f>
+        <v>4162.5</v>
+      </c>
+      <c r="I34" s="23">
         <f>I33+I16</f>
-        <v>11293.5</v>
-      </c>
-      <c r="J34" s="17">
-        <f>J33+J16</f>
-        <v>13907.5</v>
-      </c>
-      <c r="L34" s="17">
-        <f>L33+L16</f>
-        <v>15986.073999999997</v>
+        <v>8408.5</v>
+      </c>
+      <c r="J34" s="34">
+        <f>IF(J33,J20,IF(J31,J32+J19,J30))+J29</f>
+        <v>3220.5</v>
+      </c>
+      <c r="L34" s="34">
+        <f>IF(L33,L20,IF(L31,L32+L19,L30))+L29</f>
+        <v>2741.25</v>
       </c>
       <c r="M34" s="17">
         <f>M33+M16</f>
-        <v>16092.696</v>
-      </c>
-      <c r="N34" s="17">
-        <f>N33+N16</f>
-        <v>15006.847999999998</v>
-      </c>
-      <c r="O34" s="25">
-        <f>O33+O16</f>
-        <v>17961.988000000001</v>
-      </c>
-      <c r="P34" s="12"/>
+        <v>12822.696</v>
+      </c>
+      <c r="N34" s="34">
+        <f>IF(N33,N20,IF(N31,N32+N19,N30))+N29</f>
+        <v>4805</v>
+      </c>
+      <c r="O34" s="32">
+        <f>IF(O33,O20,IF(O31,O32+O19,O30))+O29</f>
+        <v>9700</v>
+      </c>
+      <c r="P34" s="20"/>
     </row>
     <row r="35" spans="6:16" x14ac:dyDescent="0.2">
-      <c r="F35" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="G35">
-        <v>15203</v>
-      </c>
-      <c r="H35">
-        <v>13221</v>
+      <c r="F35" t="s">
+        <v>43</v>
+      </c>
+      <c r="G35" s="23">
+        <f>G34+G16</f>
+        <v>12467.384615384615</v>
+      </c>
+      <c r="H35" s="23">
+        <f>H34+H16</f>
+        <v>8158.5</v>
       </c>
       <c r="I35" s="12">
         <v>14180</v>
       </c>
-      <c r="J35">
+      <c r="J35" s="17">
+        <f>J34+J16</f>
+        <v>12532.5</v>
+      </c>
+      <c r="L35" s="17">
+        <f>L34+L16</f>
+        <v>14899.073999999997</v>
+      </c>
+      <c r="N35" s="17">
+        <f>N34+N16</f>
+        <v>12996.847999999998</v>
+      </c>
+      <c r="O35" s="23">
+        <f>O34+O16</f>
+        <v>17961.988000000001</v>
+      </c>
+      <c r="P35" s="12"/>
+    </row>
+    <row r="36" spans="6:16" x14ac:dyDescent="0.2">
+      <c r="F36" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="G36">
+        <v>15203</v>
+      </c>
+      <c r="H36">
+        <v>13221</v>
+      </c>
+      <c r="I36" s="23">
+        <f>I34-I35</f>
+        <v>-5771.5</v>
+      </c>
+      <c r="J36">
         <v>12318</v>
       </c>
-      <c r="L35">
+      <c r="L36">
         <v>17567</v>
       </c>
-      <c r="P35" s="22"/>
-    </row>
-    <row r="36" spans="6:16" x14ac:dyDescent="0.2">
-      <c r="F36" t="s">
+      <c r="M36" s="23">
+        <f>M34-M35</f>
+        <v>12822.696</v>
+      </c>
+      <c r="P36" s="20"/>
+    </row>
+    <row r="37" spans="6:16" x14ac:dyDescent="0.2">
+      <c r="F37" t="s">
         <v>34</v>
       </c>
-      <c r="G36" s="25">
-        <f>G34-G35</f>
-        <v>-73.461538461539021</v>
-      </c>
-      <c r="H36" s="25">
-        <f>H34-H35</f>
-        <v>-3442.5</v>
-      </c>
-      <c r="I36" s="25">
-        <f>I34-I35</f>
-        <v>-2886.5</v>
-      </c>
-      <c r="J36" s="25">
-        <f>J34-J35</f>
-        <v>1589.5</v>
-      </c>
-      <c r="L36" s="25">
-        <f>L34-L35</f>
-        <v>-1580.9260000000031</v>
-      </c>
-      <c r="M36" s="25">
-        <f>M34-M35</f>
-        <v>16092.696</v>
-      </c>
-      <c r="N36" s="25">
-        <f>N34-N35</f>
-        <v>15006.847999999998</v>
-      </c>
-      <c r="O36" s="25">
-        <f>O34-O35</f>
+      <c r="G37" s="23">
+        <f>G35-G36</f>
+        <v>-2735.6153846153848</v>
+      </c>
+      <c r="H37" s="23">
+        <f>H35-H36</f>
+        <v>-5062.5</v>
+      </c>
+      <c r="J37" s="23">
+        <f>J35-J36</f>
+        <v>214.5</v>
+      </c>
+      <c r="L37" s="23">
+        <f>L35-L36</f>
+        <v>-2667.9260000000031</v>
+      </c>
+      <c r="N37" s="23">
+        <f>N35-N36</f>
+        <v>12996.847999999998</v>
+      </c>
+      <c r="O37" s="23">
+        <f>O35-O36</f>
         <v>17961.988000000001</v>
       </c>
-      <c r="P36" s="21"/>
-    </row>
-    <row r="37" spans="6:16" x14ac:dyDescent="0.2">
-      <c r="P37" s="21"/>
+      <c r="P37" s="19"/>
+    </row>
+    <row r="38" spans="6:16" x14ac:dyDescent="0.2">
+      <c r="P38" s="19"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G21:O21" xr:uid="{2464005F-F9F1-9D4D-B741-989E515CAA95}">
+      <formula1>"YES,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>